<commit_message>
train model I3D on MSVD
</commit_message>
<xml_diff>
--- a/Run-models.xlsx
+++ b/Run-models.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\__VC-Transformer-KG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1894223A-D768-4BED-81C9-5EAFFC01BB2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{236B0655-86A0-45C1-B20F-15A4616AD569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{FA8BBE0D-22B6-4761-9F5D-E5ADB8E48FD1}"/>
+    <workbookView xWindow="2780" yWindow="840" windowWidth="14400" windowHeight="7960" xr2:uid="{FA8BBE0D-22B6-4761-9F5D-E5ADB8E48FD1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -249,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
@@ -268,7 +268,6 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1">
       <extLst>
@@ -644,13 +643,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="13" t="s">
+      <c r="B1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1">
@@ -677,21 +676,21 @@
       <c r="A3" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="B4" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>5</v>
       </c>
     </row>
@@ -699,10 +698,10 @@
       <c r="A5" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>6</v>
       </c>
     </row>
@@ -710,10 +709,10 @@
       <c r="A6" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>7</v>
       </c>
     </row>
@@ -721,10 +720,10 @@
       <c r="A7" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="6" t="s">
         <v>8</v>
       </c>
     </row>
@@ -732,10 +731,10 @@
       <c r="A8" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>9</v>
       </c>
     </row>
@@ -743,21 +742,21 @@
       <c r="A9" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="18" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="B10" s="9" t="s">
+      <c r="A10" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
         <v>11</v>
       </c>
     </row>
@@ -776,10 +775,10 @@
       <c r="A12" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="6" t="s">
         <v>13</v>
       </c>
     </row>
@@ -787,10 +786,10 @@
       <c r="A13" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="6" t="s">
         <v>5</v>
       </c>
     </row>
@@ -798,10 +797,10 @@
       <c r="A14" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="6" t="s">
         <v>6</v>
       </c>
     </row>
@@ -809,10 +808,10 @@
       <c r="A15" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="6" t="s">
         <v>7</v>
       </c>
     </row>
@@ -820,10 +819,10 @@
       <c r="A16" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="6" t="s">
         <v>8</v>
       </c>
     </row>
@@ -831,10 +830,10 @@
       <c r="A17" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="6" t="s">
         <v>9</v>
       </c>
     </row>
@@ -842,21 +841,21 @@
       <c r="A18" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="B19" s="9" t="s">
+      <c r="A19" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="9" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
train model ResNet152+I3D on MSVD
</commit_message>
<xml_diff>
--- a/Run-models.xlsx
+++ b/Run-models.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\__VC-Transformer-KG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{236B0655-86A0-45C1-B20F-15A4616AD569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CED96EB4-98AF-4707-8275-12E457D92965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2780" yWindow="840" windowWidth="14400" windowHeight="7960" xr2:uid="{FA8BBE0D-22B6-4761-9F5D-E5ADB8E48FD1}"/>
+    <workbookView xWindow="1170" yWindow="1410" windowWidth="14400" windowHeight="7960" xr2:uid="{FA8BBE0D-22B6-4761-9F5D-E5ADB8E48FD1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -696,7 +696,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
train model ResNet152+I3D+OFeat on MSVD
</commit_message>
<xml_diff>
--- a/Run-models.xlsx
+++ b/Run-models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\__VC-Transformer-KG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CED96EB4-98AF-4707-8275-12E457D92965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{541FD1EC-379D-46B0-BF08-CD6804D17633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1170" yWindow="1410" windowWidth="14400" windowHeight="7960" xr2:uid="{FA8BBE0D-22B6-4761-9F5D-E5ADB8E48FD1}"/>
   </bookViews>
@@ -707,7 +707,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
train model ResNet152+I3D+OFeat+rel on MSVD
</commit_message>
<xml_diff>
--- a/Run-models.xlsx
+++ b/Run-models.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\__VC-Transformer-KG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{541FD1EC-379D-46B0-BF08-CD6804D17633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6325F6F1-77F5-467B-8E93-347A10E433A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1410" windowWidth="14400" windowHeight="7960" xr2:uid="{FA8BBE0D-22B6-4761-9F5D-E5ADB8E48FD1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="7610" windowHeight="10340" xr2:uid="{FA8BBE0D-22B6-4761-9F5D-E5ADB8E48FD1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -718,7 +718,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
prepare for training InceptionResNetV2+I3D on MSVD
</commit_message>
<xml_diff>
--- a/Run-models.xlsx
+++ b/Run-models.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\__VC-Transformer-KG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6325F6F1-77F5-467B-8E93-347A10E433A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFB86C33-881E-44C0-9DFB-B3B07E791EAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="7610" windowHeight="10340" xr2:uid="{FA8BBE0D-22B6-4761-9F5D-E5ADB8E48FD1}"/>
+    <workbookView xWindow="-4110" yWindow="-14510" windowWidth="25820" windowHeight="14160" xr2:uid="{FA8BBE0D-22B6-4761-9F5D-E5ADB8E48FD1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>